<commit_message>
Coach: retira «Punto débil opcional» y reparte sus ejercicios por grupo
Catálogo y plantilla embebida sin el patrón; sus ejercicios se eligen desde
Aislamiento. Las rutinas de cliente, los Excel y los ejercicios propios que
aún lo traigan pasan al patrón de su grupo o de su lista al cargarse.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B6Q4CD4Awrk5AT2kyYjdJQ
</commit_message>
<xml_diff>
--- a/coach/mi_rutina_truelift.xlsx
+++ b/coach/mi_rutina_truelift.xlsx
@@ -11,7 +11,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="7" r:id="Rc9fa6fb1bdcc4f46"/>
   </x:sheets>
   <x:definedNames>
-    <x:definedName name="PATRONES">Listas!$A$1:$A$18</x:definedName>
+    <x:definedName name="PATRONES">Listas!$A$1:$A$17</x:definedName>
     <x:definedName name="DESCANSOS">Listas!$U$1:$U$12</x:definedName>
     <x:definedName name="SISTEMAS">Listas!$V$1:$V$2</x:definedName>
     <x:definedName name="Empuje_horizontal">Listas!$C$1:$C$8</x:definedName>
@@ -21,7 +21,6 @@
     <x:definedName name="Empuje_vertical">Listas!$H$1:$H$8</x:definedName>
     <x:definedName name="Deltoide_posterior">Listas!$I$1:$I$7</x:definedName>
     <x:definedName name="Estabilidad_escapular">Listas!$J$1:$J$7</x:definedName>
-    <x:definedName name="Punto_débil_opcional">Listas!$K$1:$K$8</x:definedName>
     <x:definedName name="Rodilla">Listas!$L$1:$L$10</x:definedName>
     <x:definedName name="Unilateral">Listas!$M$1:$M$9</x:definedName>
     <x:definedName name="Bisagra">Listas!$N$1:$N$10</x:definedName>
@@ -2399,11 +2398,6 @@
           <x:t xml:space="preserve">Face pull suave en polea</x:t>
         </x:is>
       </x:c>
-      <x:c r="K1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Elevación lateral ligera en polea</x:t>
-        </x:is>
-      </x:c>
       <x:c r="L1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Sentadilla con barra</x:t>
@@ -2497,11 +2491,6 @@
           <x:t xml:space="preserve">Pull-apart con banda</x:t>
         </x:is>
       </x:c>
-      <x:c r="K2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Elevación frontal con mancuernas</x:t>
-        </x:is>
-      </x:c>
       <x:c r="L2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Hack squat en máquina</x:t>
@@ -2595,11 +2584,6 @@
           <x:t xml:space="preserve">Rotación externa con mancuerna</x:t>
         </x:is>
       </x:c>
-      <x:c r="K3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Elevación lateral ligera con mancuernas</x:t>
-        </x:is>
-      </x:c>
       <x:c r="L3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prensa 45°</x:t>
@@ -2688,9 +2672,6 @@
           <x:t xml:space="preserve">Rotación externa en polea</x:t>
         </x:is>
       </x:c>
-      <x:c r="K4" t="str">
-        <x:v>Elevación lateral en máquina</x:v>
-      </x:c>
       <x:c r="L4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prensa 45° pies medios</x:t>
@@ -2775,9 +2756,6 @@
       <x:c r="J5" t="str">
         <x:v>Elevaciones Y en banco inclinado</x:v>
       </x:c>
-      <x:c r="K5" t="str">
-        <x:v>Curl en cuerda en polea</x:v>
-      </x:c>
       <x:c r="L5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Sentadilla en Smith</x:t>
@@ -2854,9 +2832,6 @@
       <x:c r="J6" t="str">
         <x:v>Flexiones escapulares</x:v>
       </x:c>
-      <x:c r="K6" t="str">
-        <x:v>Extensión en cuerda en polea</x:v>
-      </x:c>
       <x:c r="L6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Sentadilla española</x:t>
@@ -2927,9 +2902,6 @@
       <x:c r="J7" t="str">
         <x:v>Wall slides</x:v>
       </x:c>
-      <x:c r="K7" t="str">
-        <x:v>Gemelo sentado</x:v>
-      </x:c>
       <x:c r="L7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Sentadilla goblet con mancuerna</x:t>
@@ -2989,9 +2961,6 @@
       <x:c r="H8" t="str">
         <x:v>Press landmine a una mano</x:v>
       </x:c>
-      <x:c r="K8" t="str">
-        <x:v>Crunch en máquina</x:v>
-      </x:c>
       <x:c r="L8" t="str">
         <x:v>Sentadilla frontal con barra</x:v>
       </x:c>
@@ -3056,7 +3025,7 @@
     <x:row r="10">
       <x:c r="A10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Punto débil opcional</x:t>
+          <x:t xml:space="preserve">Rodilla</x:t>
         </x:is>
       </x:c>
       <x:c r="E10" t="str">
@@ -3084,7 +3053,7 @@
     <x:row r="11">
       <x:c r="A11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Rodilla</x:t>
+          <x:t xml:space="preserve">Unilateral</x:t>
         </x:is>
       </x:c>
       <x:c r="E11" t="str">
@@ -3106,7 +3075,7 @@
     <x:row r="12">
       <x:c r="A12" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Unilateral</x:t>
+          <x:t xml:space="preserve">Bisagra</x:t>
         </x:is>
       </x:c>
       <x:c r="E12" t="str">
@@ -3128,7 +3097,7 @@
     <x:row r="13">
       <x:c r="A13" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Bisagra</x:t>
+          <x:t xml:space="preserve">Flexión de rodilla</x:t>
         </x:is>
       </x:c>
       <x:c r="E13" t="str">
@@ -3141,7 +3110,7 @@
     <x:row r="14">
       <x:c r="A14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Flexión de rodilla</x:t>
+          <x:t xml:space="preserve">Glúteo</x:t>
         </x:is>
       </x:c>
       <x:c r="E14" t="str">
@@ -3151,7 +3120,7 @@
     <x:row r="15">
       <x:c r="A15" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Glúteo</x:t>
+          <x:t xml:space="preserve">Glúteo medio</x:t>
         </x:is>
       </x:c>
       <x:c r="E15" t="str">
@@ -3161,7 +3130,7 @@
     <x:row r="16">
       <x:c r="A16" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Glúteo medio</x:t>
+          <x:t xml:space="preserve">Gemelo</x:t>
         </x:is>
       </x:c>
       <x:c r="E16" t="str">
@@ -3171,7 +3140,7 @@
     <x:row r="17">
       <x:c r="A17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Gemelo</x:t>
+          <x:t xml:space="preserve">Core</x:t>
         </x:is>
       </x:c>
       <x:c r="E17" t="str">
@@ -3179,11 +3148,6 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Core</x:t>
-        </x:is>
-      </x:c>
       <x:c r="E18" t="str">
         <x:v>Curl predicador en máquina</x:v>
       </x:c>

</xml_diff>